<commit_message>
Clean MarkOnMinds catalog and SEO leftovers
</commit_message>
<xml_diff>
--- a/storage/imports/templates/pincodes.xlsx
+++ b/storage/imports/templates/pincodes.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
   <si>
     <t>pincode</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>locality</t>
+  </si>
+  <si>
+    <t>bangalore_zone_code</t>
   </si>
   <si>
     <t>is_serviceable</t>
@@ -440,10 +443,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,6 +485,9 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -504,28 +510,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -545,31 +551,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean Medca Consultancy lab catalog
</commit_message>
<xml_diff>
--- a/storage/imports/templates/pincodes.xlsx
+++ b/storage/imports/templates/pincodes.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
   <si>
     <t>pincode</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>locality</t>
+  </si>
+  <si>
+    <t>bangalore_zone_code</t>
   </si>
   <si>
     <t>is_serviceable</t>
@@ -440,10 +443,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,6 +485,9 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -504,28 +510,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -545,31 +551,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean Karnataka Diagnostics lab catalog
</commit_message>
<xml_diff>
--- a/storage/imports/templates/pincodes.xlsx
+++ b/storage/imports/templates/pincodes.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
   <si>
     <t>pincode</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>locality</t>
+  </si>
+  <si>
+    <t>bangalore_zone_code</t>
   </si>
   <si>
     <t>is_serviceable</t>
@@ -440,10 +443,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,6 +485,9 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -504,28 +510,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -545,31 +551,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>